<commit_message>
fix(scraper): resolve HTTP 403 by adding multi-host failover, realistic browser headers, and date fallback
</commit_message>
<xml_diff>
--- a/data/Todos.xlsx
+++ b/data/Todos.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30120"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7369193B-C27D-42D1-B12D-52B994FFA874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{017B3003-76FF-4FF2-B8A0-7BA24950C5E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jornada 21" sheetId="1" r:id="rId1"/>
@@ -16,6 +16,7 @@
     <sheet name="Jornada 25" sheetId="8" r:id="rId6"/>
     <sheet name="Jornada 26" sheetId="9" r:id="rId7"/>
     <sheet name="Jornada 32" sheetId="10" r:id="rId8"/>
+    <sheet name="Todos" sheetId="11" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2742" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2898" uniqueCount="282">
   <si>
     <t>Matchday</t>
   </si>
@@ -704,6 +705,183 @@
   </si>
   <si>
     <t>22/05/2026</t>
+  </si>
+  <si>
+    <t>Jornada 15</t>
+  </si>
+  <si>
+    <t>31/07/2026</t>
+  </si>
+  <si>
+    <t>8:00 PM</t>
+  </si>
+  <si>
+    <t>North Carolina Courage</t>
+  </si>
+  <si>
+    <t>Orlando Pride</t>
+  </si>
+  <si>
+    <t>01/08/2026</t>
+  </si>
+  <si>
+    <t>Racing Louisville FC</t>
+  </si>
+  <si>
+    <t>Chicago Stars FC</t>
+  </si>
+  <si>
+    <t>6:30 PM</t>
+  </si>
+  <si>
+    <t>Kansas City Current</t>
+  </si>
+  <si>
+    <t>Angel City FC</t>
+  </si>
+  <si>
+    <t>Houston Dash</t>
+  </si>
+  <si>
+    <t>Gotham FC</t>
+  </si>
+  <si>
+    <t>8:45 PM</t>
+  </si>
+  <si>
+    <t>Bay FC</t>
+  </si>
+  <si>
+    <t>Seattle Reign FC</t>
+  </si>
+  <si>
+    <t>02/08/2026</t>
+  </si>
+  <si>
+    <t>Washington Spirit</t>
+  </si>
+  <si>
+    <t>San Diego Wave FC</t>
+  </si>
+  <si>
+    <t>Utah Royals</t>
+  </si>
+  <si>
+    <t>Portland Thorns FC</t>
+  </si>
+  <si>
+    <t>9:00 PM</t>
+  </si>
+  <si>
+    <t>Denver Summit FC</t>
+  </si>
+  <si>
+    <t>Boston Legacy FC</t>
+  </si>
+  <si>
+    <t>7:30 PM</t>
+  </si>
+  <si>
+    <t>New York City FC</t>
+  </si>
+  <si>
+    <t>Toronto FC</t>
+  </si>
+  <si>
+    <t>Jornada 20</t>
+  </si>
+  <si>
+    <t>CF Montréal</t>
+  </si>
+  <si>
+    <t>New England Revolution</t>
+  </si>
+  <si>
+    <t>D.C. United</t>
+  </si>
+  <si>
+    <t>Nashville SC</t>
+  </si>
+  <si>
+    <t>FC Cincinnati</t>
+  </si>
+  <si>
+    <t>San Jose Earthquakes</t>
+  </si>
+  <si>
+    <t>Inter Miami CF</t>
+  </si>
+  <si>
+    <t>Columbus Crew</t>
+  </si>
+  <si>
+    <t>Philadelphia Union</t>
+  </si>
+  <si>
+    <t>Atlanta United FC</t>
+  </si>
+  <si>
+    <t>Red Bull New York</t>
+  </si>
+  <si>
+    <t>Orlando City SC</t>
+  </si>
+  <si>
+    <t>Vancouver Whitecaps</t>
+  </si>
+  <si>
+    <t>LAFC</t>
+  </si>
+  <si>
+    <t>8:30 PM</t>
+  </si>
+  <si>
+    <t>Chicago Fire FC</t>
+  </si>
+  <si>
+    <t>Charlotte FC</t>
+  </si>
+  <si>
+    <t>Minnesota United FC</t>
+  </si>
+  <si>
+    <t>San Diego FC</t>
+  </si>
+  <si>
+    <t>Sporting Kansas City</t>
+  </si>
+  <si>
+    <t>Houston Dynamo FC</t>
+  </si>
+  <si>
+    <t>St. Louis CITY SC</t>
+  </si>
+  <si>
+    <t>Real Salt Lake</t>
+  </si>
+  <si>
+    <t>9:30 PM</t>
+  </si>
+  <si>
+    <t>Colorado Rapids</t>
+  </si>
+  <si>
+    <t>Austin FC</t>
+  </si>
+  <si>
+    <t>10:30 PM</t>
+  </si>
+  <si>
+    <t>LA Galaxy</t>
+  </si>
+  <si>
+    <t>FC Dallas</t>
+  </si>
+  <si>
+    <t>Portland Timbers</t>
+  </si>
+  <si>
+    <t>Seattle Sounders FC</t>
   </si>
 </sst>
 </file>
@@ -823,7 +1001,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -924,10 +1102,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
@@ -10677,28 +10851,28 @@
       <c r="H2" s="30">
         <v>1</v>
       </c>
-      <c r="I2" s="48" t="s">
+      <c r="I2" t="s">
         <v>219</v>
       </c>
-      <c r="J2" s="48" t="s">
+      <c r="J2" t="s">
         <v>27</v>
       </c>
-      <c r="K2" s="48" t="s">
+      <c r="K2" t="s">
         <v>221</v>
       </c>
-      <c r="L2" s="48" t="s">
+      <c r="L2" t="s">
         <v>85</v>
       </c>
-      <c r="M2" s="48" t="s">
+      <c r="M2" t="s">
         <v>64</v>
       </c>
-      <c r="N2" s="48" t="s">
+      <c r="N2" t="s">
         <v>74</v>
       </c>
-      <c r="O2" s="49">
-        <v>1</v>
-      </c>
-      <c r="P2" s="48">
+      <c r="O2" s="38">
+        <v>1</v>
+      </c>
+      <c r="P2">
         <v>1</v>
       </c>
     </row>
@@ -10725,28 +10899,28 @@
         <v>33</v>
       </c>
       <c r="H3" s="30"/>
-      <c r="I3" s="48" t="s">
+      <c r="I3" t="s">
         <v>219</v>
       </c>
-      <c r="J3" s="48" t="s">
+      <c r="J3" t="s">
         <v>27</v>
       </c>
-      <c r="K3" s="48" t="s">
+      <c r="K3" t="s">
         <v>221</v>
       </c>
-      <c r="L3" s="48" t="s">
+      <c r="L3" t="s">
         <v>85</v>
       </c>
-      <c r="M3" s="48" t="s">
+      <c r="M3" t="s">
         <v>82</v>
       </c>
-      <c r="N3" s="48" t="s">
+      <c r="N3" t="s">
         <v>70</v>
       </c>
-      <c r="O3" s="49" t="s">
+      <c r="O3" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="P3" s="48" t="s">
+      <c r="P3" t="s">
         <v>33</v>
       </c>
     </row>
@@ -10773,28 +10947,28 @@
         <v>33</v>
       </c>
       <c r="H4" s="30"/>
-      <c r="I4" s="48" t="s">
+      <c r="I4" t="s">
         <v>219</v>
       </c>
-      <c r="J4" s="48" t="s">
+      <c r="J4" t="s">
         <v>27</v>
       </c>
-      <c r="K4" s="48" t="s">
+      <c r="K4" t="s">
         <v>221</v>
       </c>
-      <c r="L4" s="48" t="s">
+      <c r="L4" t="s">
         <v>85</v>
       </c>
-      <c r="M4" s="48" t="s">
+      <c r="M4" t="s">
         <v>77</v>
       </c>
-      <c r="N4" s="48" t="s">
+      <c r="N4" t="s">
         <v>67</v>
       </c>
-      <c r="O4" s="49">
-        <v>1</v>
-      </c>
-      <c r="P4" s="48" t="s">
+      <c r="O4" s="38">
+        <v>1</v>
+      </c>
+      <c r="P4" t="s">
         <v>33</v>
       </c>
     </row>
@@ -10821,28 +10995,28 @@
         <v>33</v>
       </c>
       <c r="H5" s="30"/>
-      <c r="I5" s="48" t="s">
+      <c r="I5" t="s">
         <v>219</v>
       </c>
-      <c r="J5" s="48" t="s">
+      <c r="J5" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="48" t="s">
+      <c r="K5" t="s">
         <v>221</v>
       </c>
-      <c r="L5" s="48" t="s">
+      <c r="L5" t="s">
         <v>85</v>
       </c>
-      <c r="M5" s="48" t="s">
+      <c r="M5" t="s">
         <v>75</v>
       </c>
-      <c r="N5" s="48" t="s">
+      <c r="N5" t="s">
         <v>69</v>
       </c>
-      <c r="O5" s="49" t="s">
+      <c r="O5" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="P5" s="48">
+      <c r="P5">
         <v>1</v>
       </c>
     </row>
@@ -10869,28 +11043,28 @@
         <v>1</v>
       </c>
       <c r="H6" s="30"/>
-      <c r="I6" s="48" t="s">
+      <c r="I6" t="s">
         <v>219</v>
       </c>
-      <c r="J6" s="48" t="s">
+      <c r="J6" t="s">
         <v>27</v>
       </c>
-      <c r="K6" s="48" t="s">
+      <c r="K6" t="s">
         <v>221</v>
       </c>
-      <c r="L6" s="48" t="s">
+      <c r="L6" t="s">
         <v>85</v>
       </c>
-      <c r="M6" s="48" t="s">
+      <c r="M6" t="s">
         <v>68</v>
       </c>
-      <c r="N6" s="48" t="s">
+      <c r="N6" t="s">
         <v>63</v>
       </c>
-      <c r="O6" s="49">
+      <c r="O6" s="38">
         <v>2</v>
       </c>
-      <c r="P6" s="48" t="s">
+      <c r="P6" t="s">
         <v>33</v>
       </c>
     </row>
@@ -10917,28 +11091,28 @@
         <v>33</v>
       </c>
       <c r="H7" s="30"/>
-      <c r="I7" s="48" t="s">
+      <c r="I7" t="s">
         <v>219</v>
       </c>
-      <c r="J7" s="48" t="s">
+      <c r="J7" t="s">
         <v>27</v>
       </c>
-      <c r="K7" s="48" t="s">
+      <c r="K7" t="s">
         <v>221</v>
       </c>
-      <c r="L7" s="48" t="s">
+      <c r="L7" t="s">
         <v>85</v>
       </c>
-      <c r="M7" s="48" t="s">
+      <c r="M7" t="s">
         <v>79</v>
       </c>
-      <c r="N7" s="48" t="s">
+      <c r="N7" t="s">
         <v>62</v>
       </c>
-      <c r="O7" s="49" t="s">
+      <c r="O7" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="P7" s="48">
+      <c r="P7">
         <v>2</v>
       </c>
     </row>
@@ -10965,28 +11139,28 @@
         <v>2</v>
       </c>
       <c r="H8" s="30"/>
-      <c r="I8" s="48" t="s">
+      <c r="I8" t="s">
         <v>219</v>
       </c>
-      <c r="J8" s="48" t="s">
+      <c r="J8" t="s">
         <v>27</v>
       </c>
-      <c r="K8" s="48" t="s">
+      <c r="K8" t="s">
         <v>221</v>
       </c>
-      <c r="L8" s="48" t="s">
+      <c r="L8" t="s">
         <v>85</v>
       </c>
-      <c r="M8" s="48" t="s">
+      <c r="M8" t="s">
         <v>76</v>
       </c>
-      <c r="N8" s="48" t="s">
+      <c r="N8" t="s">
         <v>71</v>
       </c>
-      <c r="O8" s="49" t="s">
+      <c r="O8" s="38" t="s">
         <v>33</v>
       </c>
-      <c r="P8" s="48">
+      <c r="P8">
         <v>1</v>
       </c>
     </row>
@@ -11061,54 +11235,54 @@
         <v>1</v>
       </c>
       <c r="H10" s="30"/>
-      <c r="I10" s="48" t="s">
+      <c r="I10" t="s">
         <v>219</v>
       </c>
-      <c r="J10" s="48" t="s">
+      <c r="J10" t="s">
         <v>27</v>
       </c>
-      <c r="K10" s="48" t="s">
+      <c r="K10" t="s">
         <v>221</v>
       </c>
-      <c r="L10" s="48" t="s">
+      <c r="L10" t="s">
         <v>85</v>
       </c>
-      <c r="M10" s="48" t="s">
+      <c r="M10" t="s">
         <v>78</v>
       </c>
-      <c r="N10" s="48" t="s">
+      <c r="N10" t="s">
         <v>65</v>
       </c>
-      <c r="O10" s="49">
-        <v>1</v>
-      </c>
-      <c r="P10" s="48">
+      <c r="O10" s="38">
+        <v>1</v>
+      </c>
+      <c r="P10">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="I11" s="48" t="s">
+      <c r="I11" t="s">
         <v>219</v>
       </c>
-      <c r="J11" s="48" t="s">
+      <c r="J11" t="s">
         <v>27</v>
       </c>
-      <c r="K11" s="48" t="s">
+      <c r="K11" t="s">
         <v>221</v>
       </c>
-      <c r="L11" s="48" t="s">
+      <c r="L11" t="s">
         <v>85</v>
       </c>
-      <c r="M11" s="48" t="s">
+      <c r="M11" t="s">
         <v>73</v>
       </c>
-      <c r="N11" s="48" t="s">
+      <c r="N11" t="s">
         <v>66</v>
       </c>
-      <c r="O11" s="49">
-        <v>1</v>
-      </c>
-      <c r="P11" s="48">
+      <c r="O11" s="38">
+        <v>1</v>
+      </c>
+      <c r="P11">
         <v>2</v>
       </c>
     </row>
@@ -11158,25 +11332,25 @@
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="50" t="s">
+      <c r="A14" s="48" t="s">
         <v>219</v>
       </c>
-      <c r="B14" s="50" t="s">
+      <c r="B14" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="50" t="s">
+      <c r="C14" s="48" t="s">
         <v>222</v>
       </c>
-      <c r="D14" s="50" t="s">
+      <c r="D14" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="E14" s="50" t="s">
+      <c r="E14" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="F14" s="50" t="s">
+      <c r="F14" s="48" t="s">
         <v>50</v>
       </c>
-      <c r="G14" s="51" t="s">
+      <c r="G14" s="49" t="s">
         <v>33</v>
       </c>
       <c r="H14" s="30"/>
@@ -11206,25 +11380,25 @@
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="48" t="s">
+      <c r="A15" t="s">
         <v>219</v>
       </c>
-      <c r="B15" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="48" t="s">
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
         <v>220</v>
       </c>
-      <c r="D15" s="48" t="s">
+      <c r="D15" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="48" t="s">
+      <c r="E15" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="48" t="s">
+      <c r="F15" t="s">
         <v>52</v>
       </c>
-      <c r="G15" s="49"/>
+      <c r="G15" s="38"/>
       <c r="H15" s="30">
         <v>1</v>
       </c>
@@ -11254,25 +11428,25 @@
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" s="48" t="s">
+      <c r="A16" t="s">
         <v>219</v>
       </c>
-      <c r="B16" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="48" t="s">
+      <c r="B16" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" t="s">
         <v>220</v>
       </c>
-      <c r="D16" s="48" t="s">
+      <c r="D16" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="48" t="s">
+      <c r="E16" t="s">
         <v>36</v>
       </c>
-      <c r="F16" s="48" t="s">
+      <c r="F16" t="s">
         <v>39</v>
       </c>
-      <c r="G16" s="49">
+      <c r="G16" s="38">
         <v>1</v>
       </c>
       <c r="H16" s="30"/>
@@ -11299,25 +11473,25 @@
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="48" t="s">
+      <c r="A17" t="s">
         <v>219</v>
       </c>
-      <c r="B17" s="48" t="s">
+      <c r="B17" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="48" t="s">
+      <c r="C17" t="s">
         <v>221</v>
       </c>
-      <c r="D17" s="48" t="s">
+      <c r="D17" t="s">
         <v>38</v>
       </c>
-      <c r="E17" s="48" t="s">
+      <c r="E17" t="s">
         <v>53</v>
       </c>
-      <c r="F17" s="48" t="s">
+      <c r="F17" t="s">
         <v>40</v>
       </c>
-      <c r="G17" s="49" t="s">
+      <c r="G17" s="38" t="s">
         <v>33</v>
       </c>
       <c r="H17" s="30">
@@ -11349,25 +11523,25 @@
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="48" t="s">
+      <c r="A18" t="s">
         <v>219</v>
       </c>
-      <c r="B18" s="48" t="s">
+      <c r="B18" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="48" t="s">
+      <c r="C18" t="s">
         <v>221</v>
       </c>
-      <c r="D18" s="48" t="s">
+      <c r="D18" t="s">
         <v>41</v>
       </c>
-      <c r="E18" s="48" t="s">
+      <c r="E18" t="s">
         <v>42</v>
       </c>
-      <c r="F18" s="48" t="s">
+      <c r="F18" t="s">
         <v>56</v>
       </c>
-      <c r="G18" s="49">
+      <c r="G18" s="38">
         <v>1</v>
       </c>
       <c r="H18" s="30"/>
@@ -11490,25 +11664,25 @@
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" s="48" t="s">
+      <c r="A21" t="s">
         <v>219</v>
       </c>
-      <c r="B21" s="48" t="s">
+      <c r="B21" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="48" t="s">
+      <c r="C21" t="s">
         <v>221</v>
       </c>
-      <c r="D21" s="48" t="s">
+      <c r="D21" t="s">
         <v>35</v>
       </c>
-      <c r="E21" s="48" t="s">
+      <c r="E21" t="s">
         <v>59</v>
       </c>
-      <c r="F21" s="48" t="s">
+      <c r="F21" t="s">
         <v>44</v>
       </c>
-      <c r="G21" s="49">
+      <c r="G21" s="38">
         <v>1</v>
       </c>
       <c r="H21" s="30"/>
@@ -11535,25 +11709,25 @@
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A22" s="48" t="s">
+      <c r="A22" t="s">
         <v>219</v>
       </c>
-      <c r="B22" s="48" t="s">
+      <c r="B22" t="s">
         <v>27</v>
       </c>
-      <c r="C22" s="48" t="s">
+      <c r="C22" t="s">
         <v>221</v>
       </c>
-      <c r="D22" s="48" t="s">
+      <c r="D22" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="48" t="s">
+      <c r="E22" t="s">
         <v>47</v>
       </c>
-      <c r="F22" s="48" t="s">
+      <c r="F22" t="s">
         <v>54</v>
       </c>
-      <c r="G22" s="49">
+      <c r="G22" s="38">
         <v>2</v>
       </c>
       <c r="H22" s="30"/>
@@ -11649,25 +11823,25 @@
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="48" t="s">
+      <c r="A26" t="s">
         <v>219</v>
       </c>
-      <c r="B26" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="C26" s="48" t="s">
+      <c r="B26" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" t="s">
         <v>220</v>
       </c>
-      <c r="D26" s="48" t="s">
+      <c r="D26" t="s">
         <v>80</v>
       </c>
-      <c r="E26" s="48" t="s">
+      <c r="E26" t="s">
         <v>124</v>
       </c>
-      <c r="F26" s="48" t="s">
+      <c r="F26" t="s">
         <v>115</v>
       </c>
-      <c r="G26" s="49" t="s">
+      <c r="G26" s="38" t="s">
         <v>33</v>
       </c>
       <c r="H26" s="30"/>
@@ -11707,25 +11881,25 @@
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A28" s="48" t="s">
+      <c r="A28" t="s">
         <v>219</v>
       </c>
-      <c r="B28" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28" s="48" t="s">
+      <c r="B28" t="s">
+        <v>12</v>
+      </c>
+      <c r="C28" t="s">
         <v>220</v>
       </c>
-      <c r="D28" s="48" t="s">
+      <c r="D28" t="s">
         <v>80</v>
       </c>
-      <c r="E28" s="48" t="s">
+      <c r="E28" t="s">
         <v>112</v>
       </c>
-      <c r="F28" s="48" t="s">
+      <c r="F28" t="s">
         <v>120</v>
       </c>
-      <c r="G28" s="49" t="s">
+      <c r="G28" s="38" t="s">
         <v>33</v>
       </c>
       <c r="H28" s="30"/>
@@ -11736,25 +11910,25 @@
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A29" s="48" t="s">
+      <c r="A29" t="s">
         <v>219</v>
       </c>
-      <c r="B29" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="C29" s="48" t="s">
+      <c r="B29" t="s">
+        <v>12</v>
+      </c>
+      <c r="C29" t="s">
         <v>220</v>
       </c>
-      <c r="D29" s="48" t="s">
+      <c r="D29" t="s">
         <v>80</v>
       </c>
-      <c r="E29" s="48" t="s">
+      <c r="E29" t="s">
         <v>133</v>
       </c>
-      <c r="F29" s="48" t="s">
+      <c r="F29" t="s">
         <v>122</v>
       </c>
-      <c r="G29" s="49" t="s">
+      <c r="G29" s="38" t="s">
         <v>33</v>
       </c>
       <c r="H29" s="30"/>
@@ -11765,25 +11939,25 @@
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A30" s="48" t="s">
+      <c r="A30" t="s">
         <v>219</v>
       </c>
-      <c r="B30" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="C30" s="48" t="s">
+      <c r="B30" t="s">
+        <v>12</v>
+      </c>
+      <c r="C30" t="s">
         <v>220</v>
       </c>
-      <c r="D30" s="48" t="s">
+      <c r="D30" t="s">
         <v>80</v>
       </c>
-      <c r="E30" s="48" t="s">
+      <c r="E30" t="s">
         <v>125</v>
       </c>
-      <c r="F30" s="48" t="s">
+      <c r="F30" t="s">
         <v>113</v>
       </c>
-      <c r="G30" s="49" t="s">
+      <c r="G30" s="38" t="s">
         <v>33</v>
       </c>
       <c r="H30" s="30"/>
@@ -11823,25 +11997,25 @@
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A32" s="48" t="s">
+      <c r="A32" t="s">
         <v>219</v>
       </c>
-      <c r="B32" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="C32" s="48" t="s">
+      <c r="B32" t="s">
+        <v>12</v>
+      </c>
+      <c r="C32" t="s">
         <v>220</v>
       </c>
-      <c r="D32" s="48" t="s">
+      <c r="D32" t="s">
         <v>80</v>
       </c>
-      <c r="E32" s="48" t="s">
+      <c r="E32" t="s">
         <v>131</v>
       </c>
-      <c r="F32" s="48" t="s">
+      <c r="F32" t="s">
         <v>126</v>
       </c>
-      <c r="G32" s="49">
+      <c r="G32" s="38">
         <v>1</v>
       </c>
       <c r="H32" s="30"/>
@@ -11852,25 +12026,25 @@
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" s="48" t="s">
+      <c r="A33" t="s">
         <v>219</v>
       </c>
-      <c r="B33" s="48" t="s">
-        <v>12</v>
-      </c>
-      <c r="C33" s="48" t="s">
+      <c r="B33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" t="s">
         <v>220</v>
       </c>
-      <c r="D33" s="48" t="s">
+      <c r="D33" t="s">
         <v>80</v>
       </c>
-      <c r="E33" s="48" t="s">
+      <c r="E33" t="s">
         <v>130</v>
       </c>
-      <c r="F33" s="48" t="s">
+      <c r="F33" t="s">
         <v>118</v>
       </c>
-      <c r="G33" s="49" t="s">
+      <c r="G33" s="38" t="s">
         <v>33</v>
       </c>
       <c r="H33" s="30"/>
@@ -11910,25 +12084,25 @@
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="48" t="s">
+      <c r="A35" t="s">
         <v>219</v>
       </c>
-      <c r="B35" s="48" t="s">
+      <c r="B35" t="s">
         <v>27</v>
       </c>
-      <c r="C35" s="48" t="s">
+      <c r="C35" t="s">
         <v>221</v>
       </c>
-      <c r="D35" s="48" t="s">
+      <c r="D35" t="s">
         <v>80</v>
       </c>
-      <c r="E35" s="48" t="s">
+      <c r="E35" t="s">
         <v>132</v>
       </c>
-      <c r="F35" s="48" t="s">
+      <c r="F35" t="s">
         <v>128</v>
       </c>
-      <c r="G35" s="49" t="s">
+      <c r="G35" s="38" t="s">
         <v>33</v>
       </c>
       <c r="H35" s="30"/>
@@ -11942,4 +12116,604 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01955996-BEC5-41A2-ACA9-E5AD846E62BF}">
+  <dimension ref="B2:P17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="3.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3.28515625" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" s="2"/>
+      <c r="J2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L2" t="s">
+        <v>2</v>
+      </c>
+      <c r="M2" t="s">
+        <v>3</v>
+      </c>
+      <c r="N2" t="s">
+        <v>4</v>
+      </c>
+      <c r="O2" t="s">
+        <v>5</v>
+      </c>
+      <c r="P2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>223</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>224</v>
+      </c>
+      <c r="E3" t="s">
+        <v>225</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="H3" s="32">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2"/>
+      <c r="J3" t="s">
+        <v>250</v>
+      </c>
+      <c r="K3" t="s">
+        <v>7</v>
+      </c>
+      <c r="L3" t="s">
+        <v>224</v>
+      </c>
+      <c r="M3" t="s">
+        <v>247</v>
+      </c>
+      <c r="N3" t="s">
+        <v>248</v>
+      </c>
+      <c r="O3" t="s">
+        <v>249</v>
+      </c>
+      <c r="P3" s="38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>223</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>228</v>
+      </c>
+      <c r="E4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="H4" s="32">
+        <v>1</v>
+      </c>
+      <c r="I4" s="2"/>
+      <c r="J4" t="s">
+        <v>250</v>
+      </c>
+      <c r="K4" t="s">
+        <v>12</v>
+      </c>
+      <c r="L4" t="s">
+        <v>228</v>
+      </c>
+      <c r="M4" t="s">
+        <v>247</v>
+      </c>
+      <c r="N4" t="s">
+        <v>251</v>
+      </c>
+      <c r="O4" t="s">
+        <v>252</v>
+      </c>
+      <c r="P4" s="38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>223</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>228</v>
+      </c>
+      <c r="E5" t="s">
+        <v>231</v>
+      </c>
+      <c r="F5" t="s">
+        <v>232</v>
+      </c>
+      <c r="G5" t="s">
+        <v>233</v>
+      </c>
+      <c r="H5" s="38">
+        <v>1</v>
+      </c>
+      <c r="I5" s="2"/>
+      <c r="J5" t="s">
+        <v>250</v>
+      </c>
+      <c r="K5" t="s">
+        <v>12</v>
+      </c>
+      <c r="L5" t="s">
+        <v>228</v>
+      </c>
+      <c r="M5" t="s">
+        <v>247</v>
+      </c>
+      <c r="N5" t="s">
+        <v>253</v>
+      </c>
+      <c r="O5" t="s">
+        <v>254</v>
+      </c>
+      <c r="P5" s="38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>223</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>228</v>
+      </c>
+      <c r="E6" t="s">
+        <v>225</v>
+      </c>
+      <c r="F6" t="s">
+        <v>234</v>
+      </c>
+      <c r="G6" t="s">
+        <v>235</v>
+      </c>
+      <c r="H6" s="38">
+        <v>2</v>
+      </c>
+      <c r="I6" s="2"/>
+      <c r="J6" t="s">
+        <v>250</v>
+      </c>
+      <c r="K6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L6" t="s">
+        <v>228</v>
+      </c>
+      <c r="M6" t="s">
+        <v>247</v>
+      </c>
+      <c r="N6" t="s">
+        <v>255</v>
+      </c>
+      <c r="O6" t="s">
+        <v>256</v>
+      </c>
+      <c r="P6" s="38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>223</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>228</v>
+      </c>
+      <c r="E7" t="s">
+        <v>236</v>
+      </c>
+      <c r="F7" t="s">
+        <v>237</v>
+      </c>
+      <c r="G7" t="s">
+        <v>238</v>
+      </c>
+      <c r="H7" s="38">
+        <v>2</v>
+      </c>
+      <c r="I7" s="2"/>
+      <c r="J7" t="s">
+        <v>250</v>
+      </c>
+      <c r="K7" t="s">
+        <v>12</v>
+      </c>
+      <c r="L7" t="s">
+        <v>228</v>
+      </c>
+      <c r="M7" t="s">
+        <v>247</v>
+      </c>
+      <c r="N7" t="s">
+        <v>257</v>
+      </c>
+      <c r="O7" t="s">
+        <v>258</v>
+      </c>
+      <c r="P7" s="38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>223</v>
+      </c>
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" t="s">
+        <v>239</v>
+      </c>
+      <c r="E8" t="s">
+        <v>80</v>
+      </c>
+      <c r="F8" t="s">
+        <v>240</v>
+      </c>
+      <c r="G8" t="s">
+        <v>241</v>
+      </c>
+      <c r="H8" s="38">
+        <v>1</v>
+      </c>
+      <c r="I8" s="2"/>
+      <c r="J8" t="s">
+        <v>250</v>
+      </c>
+      <c r="K8" t="s">
+        <v>12</v>
+      </c>
+      <c r="L8" t="s">
+        <v>228</v>
+      </c>
+      <c r="M8" t="s">
+        <v>247</v>
+      </c>
+      <c r="N8" t="s">
+        <v>259</v>
+      </c>
+      <c r="O8" t="s">
+        <v>260</v>
+      </c>
+      <c r="P8" s="38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>223</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
+        <v>239</v>
+      </c>
+      <c r="E9" t="s">
+        <v>208</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="H9" s="32">
+        <v>1</v>
+      </c>
+      <c r="I9" s="2"/>
+      <c r="J9" t="s">
+        <v>250</v>
+      </c>
+      <c r="K9" t="s">
+        <v>12</v>
+      </c>
+      <c r="L9" t="s">
+        <v>228</v>
+      </c>
+      <c r="M9" t="s">
+        <v>247</v>
+      </c>
+      <c r="N9" t="s">
+        <v>261</v>
+      </c>
+      <c r="O9" t="s">
+        <v>262</v>
+      </c>
+      <c r="P9" s="38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>223</v>
+      </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" t="s">
+        <v>239</v>
+      </c>
+      <c r="E10" t="s">
+        <v>244</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="H10" s="32">
+        <v>1</v>
+      </c>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="P10" s="32">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="I11" s="2"/>
+      <c r="J11" t="s">
+        <v>250</v>
+      </c>
+      <c r="K11" t="s">
+        <v>12</v>
+      </c>
+      <c r="L11" t="s">
+        <v>228</v>
+      </c>
+      <c r="M11" t="s">
+        <v>265</v>
+      </c>
+      <c r="N11" t="s">
+        <v>266</v>
+      </c>
+      <c r="O11" t="s">
+        <v>267</v>
+      </c>
+      <c r="P11" s="38" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="I12" s="2"/>
+      <c r="J12" t="s">
+        <v>250</v>
+      </c>
+      <c r="K12" t="s">
+        <v>12</v>
+      </c>
+      <c r="L12" t="s">
+        <v>228</v>
+      </c>
+      <c r="M12" t="s">
+        <v>265</v>
+      </c>
+      <c r="N12" t="s">
+        <v>268</v>
+      </c>
+      <c r="O12" t="s">
+        <v>269</v>
+      </c>
+      <c r="P12" s="38" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="I13" s="2"/>
+      <c r="J13" t="s">
+        <v>250</v>
+      </c>
+      <c r="K13" t="s">
+        <v>12</v>
+      </c>
+      <c r="L13" t="s">
+        <v>228</v>
+      </c>
+      <c r="M13" t="s">
+        <v>265</v>
+      </c>
+      <c r="N13" t="s">
+        <v>270</v>
+      </c>
+      <c r="O13" t="s">
+        <v>271</v>
+      </c>
+      <c r="P13" s="38" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="I14" s="2"/>
+      <c r="J14" t="s">
+        <v>250</v>
+      </c>
+      <c r="K14" t="s">
+        <v>12</v>
+      </c>
+      <c r="L14" t="s">
+        <v>228</v>
+      </c>
+      <c r="M14" t="s">
+        <v>265</v>
+      </c>
+      <c r="N14" t="s">
+        <v>272</v>
+      </c>
+      <c r="O14" t="s">
+        <v>273</v>
+      </c>
+      <c r="P14" s="38" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="I15" s="2"/>
+      <c r="J15" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="P15" s="32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="I16" s="2"/>
+      <c r="J16" t="s">
+        <v>250</v>
+      </c>
+      <c r="K16" t="s">
+        <v>12</v>
+      </c>
+      <c r="L16" t="s">
+        <v>228</v>
+      </c>
+      <c r="M16" t="s">
+        <v>277</v>
+      </c>
+      <c r="N16" t="s">
+        <v>278</v>
+      </c>
+      <c r="O16" t="s">
+        <v>279</v>
+      </c>
+      <c r="P16" s="38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="9:16" x14ac:dyDescent="0.25">
+      <c r="I17" s="2"/>
+      <c r="J17" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="O17" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="P17" s="32">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>